<commit_message>
Update business analysis file
</commit_message>
<xml_diff>
--- a/public/projects/business-analysis-revised.xlsx
+++ b/public/projects/business-analysis-revised.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dhanu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{139DBDDC-2488-409C-9B10-4EBC8EED23D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79D46D2E-EF42-414C-8AC5-7798AA1526CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5480" yWindow="2280" windowWidth="15820" windowHeight="11170" tabRatio="1000" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5480" yWindow="2280" windowWidth="15820" windowHeight="11170" tabRatio="1000" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="5.ID" sheetId="4" state="veryHidden" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="173">
   <si>
     <t>Name</t>
   </si>
@@ -404,65 +404,6 @@
   </si>
   <si>
     <t xml:space="preserve">FOOD TRUCK </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">2.  Create a pivot table selecting </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Existing Worksheet</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> at </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">location </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>D2</t>
-    </r>
-  </si>
-  <si>
-    <t>3. Confirm that there is no data from earlier than Jan 2019, and then remove that line</t>
-  </si>
-  <si>
-    <t>5. Insert the trend line for 2022 and include the equation</t>
-  </si>
-  <si>
-    <t>1. Copy your data set to columns A and B, leave the labels</t>
-  </si>
-  <si>
-    <t>4. Create a Pivot Graph that looks like the one given in the Project instructions on Csepub</t>
   </si>
   <si>
     <t>Variable  Expense: Donut</t>
@@ -1773,7 +1714,7 @@
     <xf numFmtId="9" fontId="25" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="194">
+  <cellXfs count="193">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2025,9 +1966,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2110,6 +2048,22 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="41" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="23" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="36" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="23" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2118,22 +2072,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="41" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="23" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="36" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="23" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -5601,13 +5539,13 @@
     </row>
     <row r="2" spans="1:24" ht="15.5">
       <c r="A2" s="9"/>
-      <c r="B2" s="140"/>
+      <c r="B2" s="139"/>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
     </row>
     <row r="3" spans="1:24" ht="15.5">
       <c r="A3" s="10"/>
-      <c r="B3" s="140"/>
+      <c r="B3" s="139"/>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
     </row>
@@ -5616,11 +5554,11 @@
       <c r="F4" s="113"/>
     </row>
     <row r="5" spans="1:24" s="112" customFormat="1" ht="15" thickBot="1">
-      <c r="E5" s="161" t="s">
-        <v>126</v>
+      <c r="E5" s="160" t="s">
+        <v>121</v>
       </c>
       <c r="F5" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
@@ -5651,7 +5589,7 @@
       <c r="C6" s="116" t="s">
         <v>107</v>
       </c>
-      <c r="E6" s="162" t="s">
+      <c r="E6" s="161" t="s">
         <v>110</v>
       </c>
       <c r="F6">
@@ -5662,13 +5600,13 @@
       <c r="A7" s="117" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="141" t="s">
+      <c r="B7" s="140" t="s">
         <v>108</v>
       </c>
       <c r="C7" s="118">
         <v>2.99</v>
       </c>
-      <c r="E7" s="162" t="s">
+      <c r="E7" s="161" t="s">
         <v>108</v>
       </c>
       <c r="F7">
@@ -5679,13 +5617,13 @@
       <c r="A8" s="117" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="141" t="s">
+      <c r="B8" s="140" t="s">
         <v>109</v>
       </c>
       <c r="C8" s="118">
         <v>2.5</v>
       </c>
-      <c r="E8" s="162" t="s">
+      <c r="E8" s="161" t="s">
         <v>109</v>
       </c>
       <c r="F8">
@@ -5696,14 +5634,14 @@
       <c r="A9" s="119" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="141" t="s">
-        <v>119</v>
+      <c r="B9" s="140" t="s">
+        <v>114</v>
       </c>
       <c r="C9" s="13">
         <v>0.5</v>
       </c>
-      <c r="E9" s="162" t="s">
-        <v>120</v>
+      <c r="E9" s="161" t="s">
+        <v>115</v>
       </c>
       <c r="F9">
         <v>0.5</v>
@@ -5713,14 +5651,14 @@
       <c r="A10" s="119" t="s">
         <v>111</v>
       </c>
-      <c r="B10" s="141" t="s">
-        <v>119</v>
+      <c r="B10" s="140" t="s">
+        <v>114</v>
       </c>
       <c r="C10" s="13">
         <v>0.1</v>
       </c>
-      <c r="E10" s="162" t="s">
-        <v>119</v>
+      <c r="E10" s="161" t="s">
+        <v>114</v>
       </c>
       <c r="F10">
         <v>0.6</v>
@@ -5730,14 +5668,14 @@
       <c r="A11" s="119" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="141" t="s">
+      <c r="B11" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C11" s="13">
         <v>300</v>
       </c>
-      <c r="E11" s="162" t="s">
-        <v>127</v>
+      <c r="E11" s="161" t="s">
+        <v>122</v>
       </c>
       <c r="F11">
         <v>5806.59</v>
@@ -5747,7 +5685,7 @@
       <c r="A12" s="119" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="141" t="s">
+      <c r="B12" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C12" s="13">
@@ -5758,7 +5696,7 @@
       <c r="A13" s="119" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="141" t="s">
+      <c r="B13" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C13" s="13">
@@ -5769,8 +5707,8 @@
       <c r="A14" s="119" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="141" t="s">
-        <v>120</v>
+      <c r="B14" s="140" t="s">
+        <v>115</v>
       </c>
       <c r="C14" s="13">
         <v>0.35</v>
@@ -5780,8 +5718,8 @@
       <c r="A15" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="141" t="s">
-        <v>120</v>
+      <c r="B15" s="140" t="s">
+        <v>115</v>
       </c>
       <c r="C15" s="13">
         <v>0.15</v>
@@ -5791,7 +5729,7 @@
       <c r="A16" s="119" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="141" t="s">
+      <c r="B16" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C16" s="13">
@@ -5802,7 +5740,7 @@
       <c r="A17" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="141" t="s">
+      <c r="B17" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C17" s="13">
@@ -5813,7 +5751,7 @@
       <c r="A18" s="119" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="141" t="s">
+      <c r="B18" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C18" s="13">
@@ -5824,7 +5762,7 @@
       <c r="A19" s="119" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="141" t="s">
+      <c r="B19" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C19" s="13">
@@ -5835,7 +5773,7 @@
       <c r="A20" s="119" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="141" t="s">
+      <c r="B20" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C20" s="13">
@@ -5846,7 +5784,7 @@
       <c r="A21" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="141" t="s">
+      <c r="B21" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C21" s="13">
@@ -5857,7 +5795,7 @@
       <c r="A22" s="119" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="141" t="s">
+      <c r="B22" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C22" s="13">
@@ -5868,7 +5806,7 @@
       <c r="A23" s="119" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="141" t="s">
+      <c r="B23" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C23" s="13">
@@ -5879,7 +5817,7 @@
       <c r="A24" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="141" t="s">
+      <c r="B24" s="140" t="s">
         <v>110</v>
       </c>
       <c r="C24" s="12">
@@ -5898,21 +5836,21 @@
       <c r="A26" s="122"/>
     </row>
     <row r="28" spans="1:5">
-      <c r="B28" s="142"/>
+      <c r="B28" s="141"/>
       <c r="C28" s="15"/>
     </row>
     <row r="29" spans="1:5" ht="16" thickBot="1">
       <c r="A29" s="123" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="142"/>
+      <c r="B29" s="141"/>
       <c r="C29" s="15"/>
     </row>
     <row r="30" spans="1:5" ht="21">
       <c r="A30" s="124" t="s">
         <v>101</v>
       </c>
-      <c r="B30" s="143"/>
+      <c r="B30" s="142"/>
       <c r="D30" s="125"/>
       <c r="E30" s="125"/>
     </row>
@@ -5944,7 +5882,7 @@
       <c r="A34" s="107" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="144">
+      <c r="B34" s="143">
         <v>0.22</v>
       </c>
       <c r="C34" s="77"/>
@@ -5955,7 +5893,7 @@
       <c r="A35" s="107" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="145">
+      <c r="B35" s="144">
         <v>0.26</v>
       </c>
     </row>
@@ -5963,14 +5901,14 @@
       <c r="A36" s="127" t="s">
         <v>99</v>
       </c>
-      <c r="B36" s="146"/>
+      <c r="B36" s="145"/>
       <c r="C36" s="46"/>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" s="128" t="s">
         <v>82</v>
       </c>
-      <c r="B37" s="147">
+      <c r="B37" s="146">
         <v>4350</v>
       </c>
     </row>
@@ -5978,7 +5916,7 @@
       <c r="A38" s="128" t="s">
         <v>83</v>
       </c>
-      <c r="B38" s="148">
+      <c r="B38" s="147">
         <v>0.32</v>
       </c>
       <c r="C38" s="47"/>
@@ -5988,7 +5926,7 @@
       <c r="A39" s="129" t="s">
         <v>84</v>
       </c>
-      <c r="B39" s="145">
+      <c r="B39" s="144">
         <v>0.22</v>
       </c>
     </row>
@@ -5996,7 +5934,7 @@
       <c r="A40" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="B40" s="149" t="s">
+      <c r="B40" s="148" t="s">
         <v>102</v>
       </c>
       <c r="C40" s="132"/>
@@ -6006,7 +5944,7 @@
       <c r="A41" s="49" t="s">
         <v>103</v>
       </c>
-      <c r="B41" s="150">
+      <c r="B41" s="149">
         <v>0.2</v>
       </c>
       <c r="C41" s="15"/>
@@ -6015,7 +5953,7 @@
       <c r="A42" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="B42" s="150">
+      <c r="B42" s="149">
         <v>0.55000000000000004</v>
       </c>
       <c r="C42" s="15"/>
@@ -6024,64 +5962,64 @@
       <c r="A43" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="B43" s="151">
+      <c r="B43" s="150">
         <v>0.25</v>
       </c>
       <c r="C43" s="15"/>
     </row>
     <row r="44" spans="1:7">
       <c r="A44" s="121"/>
-      <c r="B44" s="142"/>
+      <c r="B44" s="141"/>
       <c r="C44" s="15"/>
     </row>
     <row r="45" spans="1:7">
       <c r="A45" s="121"/>
-      <c r="B45" s="142"/>
+      <c r="B45" s="141"/>
       <c r="C45" s="15"/>
     </row>
     <row r="46" spans="1:7">
       <c r="A46" s="121"/>
-      <c r="B46" s="142"/>
+      <c r="B46" s="141"/>
       <c r="C46" s="15"/>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" s="121"/>
-      <c r="B47" s="142"/>
+      <c r="B47" s="141"/>
       <c r="C47" s="15"/>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" s="16"/>
-      <c r="B48" s="142"/>
+      <c r="B48" s="141"/>
       <c r="C48" s="15"/>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="121"/>
-      <c r="B49" s="142"/>
+      <c r="B49" s="141"/>
       <c r="C49" s="15"/>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="16"/>
-      <c r="B50" s="142"/>
+      <c r="B50" s="141"/>
       <c r="C50" s="15"/>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="121"/>
-      <c r="B51" s="142"/>
+      <c r="B51" s="141"/>
       <c r="C51" s="15"/>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" s="121"/>
-      <c r="B52" s="142"/>
+      <c r="B52" s="141"/>
       <c r="C52" s="15"/>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="121"/>
-      <c r="B53" s="142"/>
+      <c r="B53" s="141"/>
       <c r="C53" s="15"/>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="121"/>
-      <c r="B54" s="142"/>
+      <c r="B54" s="141"/>
       <c r="C54" s="15"/>
     </row>
     <row r="61" spans="1:3">
@@ -6100,7 +6038,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0326AEDA-F2D7-49C4-96A6-D7924DCB044B}">
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
     <col min="4" max="4" width="13.1796875" bestFit="1" customWidth="1"/>
@@ -6109,7 +6047,7 @@
     <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="16" thickBot="1">
+    <row r="1" spans="1:8" ht="16" thickBot="1">
       <c r="A1" s="17" t="s">
         <v>35</v>
       </c>
@@ -6117,58 +6055,52 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15.5">
-      <c r="A2" s="159">
+    <row r="2" spans="1:8" ht="15.5">
+      <c r="A2" s="158">
         <v>43831</v>
       </c>
       <c r="B2" s="104">
         <v>2395</v>
       </c>
-      <c r="D2" s="161" t="s">
-        <v>131</v>
-      </c>
-      <c r="E2" s="161" t="s">
-        <v>132</v>
-      </c>
-      <c r="P2" s="139" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="15.5">
-      <c r="A3" s="159">
+      <c r="D2" s="160" t="s">
+        <v>126</v>
+      </c>
+      <c r="E2" s="160" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15.5">
+      <c r="A3" s="158">
         <v>43862</v>
       </c>
       <c r="B3" s="104">
         <v>2584</v>
       </c>
-      <c r="D3" s="161" t="s">
-        <v>126</v>
+      <c r="D3" s="160" t="s">
+        <v>121</v>
       </c>
       <c r="E3" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="G3" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="H3" t="s">
-        <v>127</v>
-      </c>
-      <c r="P3" s="139" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="15.5">
-      <c r="A4" s="159">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.5">
+      <c r="A4" s="158">
         <v>43891</v>
       </c>
       <c r="B4" s="104">
         <v>2681</v>
       </c>
-      <c r="D4" s="162" t="s">
-        <v>133</v>
+      <c r="D4" s="161" t="s">
+        <v>128</v>
       </c>
       <c r="E4">
         <v>2395</v>
@@ -6182,19 +6114,16 @@
       <c r="H4">
         <v>7305</v>
       </c>
-      <c r="P4" s="139" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="15.5">
-      <c r="A5" s="159">
+    </row>
+    <row r="5" spans="1:8" ht="15.5">
+      <c r="A5" s="158">
         <v>43922</v>
       </c>
       <c r="B5" s="104">
         <v>3002</v>
       </c>
-      <c r="D5" s="162" t="s">
-        <v>134</v>
+      <c r="D5" s="161" t="s">
+        <v>129</v>
       </c>
       <c r="E5">
         <v>2584</v>
@@ -6208,19 +6137,16 @@
       <c r="H5">
         <v>8250</v>
       </c>
-      <c r="P5" s="139" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="15.5">
-      <c r="A6" s="159">
+    </row>
+    <row r="6" spans="1:8" ht="15.5">
+      <c r="A6" s="158">
         <v>43952</v>
       </c>
       <c r="B6" s="104">
         <v>3473</v>
       </c>
-      <c r="D6" s="162" t="s">
-        <v>135</v>
+      <c r="D6" s="161" t="s">
+        <v>130</v>
       </c>
       <c r="E6">
         <v>2681</v>
@@ -6234,19 +6160,16 @@
       <c r="H6">
         <v>8441</v>
       </c>
-      <c r="P6" s="139" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="15.5">
-      <c r="A7" s="159">
+    </row>
+    <row r="7" spans="1:8" ht="15.5">
+      <c r="A7" s="158">
         <v>43983</v>
       </c>
       <c r="B7" s="104">
         <v>3358</v>
       </c>
-      <c r="D7" s="162" t="s">
-        <v>136</v>
+      <c r="D7" s="161" t="s">
+        <v>131</v>
       </c>
       <c r="E7">
         <v>3002</v>
@@ -6261,15 +6184,15 @@
         <v>9419</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15.5">
-      <c r="A8" s="159">
+    <row r="8" spans="1:8" ht="15.5">
+      <c r="A8" s="158">
         <v>44013</v>
       </c>
       <c r="B8" s="104">
         <v>1201</v>
       </c>
-      <c r="D8" s="162" t="s">
-        <v>137</v>
+      <c r="D8" s="161" t="s">
+        <v>132</v>
       </c>
       <c r="E8">
         <v>3473</v>
@@ -6284,15 +6207,15 @@
         <v>10787</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="15.5">
-      <c r="A9" s="159">
+    <row r="9" spans="1:8" ht="15.5">
+      <c r="A9" s="158">
         <v>44044</v>
       </c>
       <c r="B9" s="104">
         <v>2549</v>
       </c>
-      <c r="D9" s="162" t="s">
-        <v>138</v>
+      <c r="D9" s="161" t="s">
+        <v>133</v>
       </c>
       <c r="E9">
         <v>3358</v>
@@ -6307,15 +6230,15 @@
         <v>10760</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="15.5">
-      <c r="A10" s="159">
+    <row r="10" spans="1:8" ht="15.5">
+      <c r="A10" s="158">
         <v>44075</v>
       </c>
       <c r="B10" s="104">
         <v>3012</v>
       </c>
-      <c r="D10" s="162" t="s">
-        <v>139</v>
+      <c r="D10" s="161" t="s">
+        <v>134</v>
       </c>
       <c r="E10">
         <v>1201</v>
@@ -6330,15 +6253,15 @@
         <v>6810</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="15.5">
-      <c r="A11" s="159">
+    <row r="11" spans="1:8" ht="15.5">
+      <c r="A11" s="158">
         <v>44105</v>
       </c>
       <c r="B11" s="104">
         <v>3561</v>
       </c>
-      <c r="D11" s="162" t="s">
-        <v>140</v>
+      <c r="D11" s="161" t="s">
+        <v>135</v>
       </c>
       <c r="E11">
         <v>2549</v>
@@ -6353,15 +6276,15 @@
         <v>8899</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="15.5">
-      <c r="A12" s="159">
+    <row r="12" spans="1:8" ht="15.5">
+      <c r="A12" s="158">
         <v>44136</v>
       </c>
       <c r="B12" s="104">
         <v>3432</v>
       </c>
-      <c r="D12" s="162" t="s">
-        <v>141</v>
+      <c r="D12" s="161" t="s">
+        <v>136</v>
       </c>
       <c r="E12">
         <v>3012</v>
@@ -6376,15 +6299,15 @@
         <v>9381</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="15.5">
-      <c r="A13" s="159">
+    <row r="13" spans="1:8" ht="15.5">
+      <c r="A13" s="158">
         <v>44166</v>
       </c>
       <c r="B13" s="105">
         <v>4515</v>
       </c>
-      <c r="D13" s="162" t="s">
-        <v>142</v>
+      <c r="D13" s="161" t="s">
+        <v>137</v>
       </c>
       <c r="E13">
         <v>3561</v>
@@ -6399,15 +6322,15 @@
         <v>11863</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="15.5">
-      <c r="A14" s="159">
+    <row r="14" spans="1:8" ht="15.5">
+      <c r="A14" s="158">
         <v>44197</v>
       </c>
       <c r="B14" s="104">
         <v>2434</v>
       </c>
-      <c r="D14" s="162" t="s">
-        <v>143</v>
+      <c r="D14" s="161" t="s">
+        <v>138</v>
       </c>
       <c r="E14">
         <v>3432</v>
@@ -6422,15 +6345,15 @@
         <v>12398</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="15.5">
-      <c r="A15" s="159">
+    <row r="15" spans="1:8" ht="15.5">
+      <c r="A15" s="158">
         <v>44228</v>
       </c>
       <c r="B15" s="104">
         <v>2627</v>
       </c>
-      <c r="D15" s="162" t="s">
-        <v>144</v>
+      <c r="D15" s="161" t="s">
+        <v>139</v>
       </c>
       <c r="E15">
         <v>4515</v>
@@ -6445,15 +6368,15 @@
         <v>16020</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="15.5">
-      <c r="A16" s="159">
+    <row r="16" spans="1:8" ht="15.5">
+      <c r="A16" s="158">
         <v>44256</v>
       </c>
       <c r="B16" s="104">
         <v>2710</v>
       </c>
-      <c r="D16" s="162" t="s">
-        <v>127</v>
+      <c r="D16" s="161" t="s">
+        <v>122</v>
       </c>
       <c r="E16">
         <v>35763</v>
@@ -6469,7 +6392,7 @@
       </c>
     </row>
     <row r="17" spans="1:2" ht="15.5">
-      <c r="A17" s="159">
+      <c r="A17" s="158">
         <v>44287</v>
       </c>
       <c r="B17" s="104">
@@ -6477,7 +6400,7 @@
       </c>
     </row>
     <row r="18" spans="1:2" ht="15.5">
-      <c r="A18" s="159">
+      <c r="A18" s="158">
         <v>44317</v>
       </c>
       <c r="B18" s="104">
@@ -6485,7 +6408,7 @@
       </c>
     </row>
     <row r="19" spans="1:2" ht="15.5">
-      <c r="A19" s="159">
+      <c r="A19" s="158">
         <v>44348</v>
       </c>
       <c r="B19" s="104">
@@ -6493,7 +6416,7 @@
       </c>
     </row>
     <row r="20" spans="1:2" ht="15.5">
-      <c r="A20" s="159">
+      <c r="A20" s="158">
         <v>44378</v>
       </c>
       <c r="B20" s="104">
@@ -6501,7 +6424,7 @@
       </c>
     </row>
     <row r="21" spans="1:2" ht="15.5">
-      <c r="A21" s="159">
+      <c r="A21" s="158">
         <v>44409</v>
       </c>
       <c r="B21" s="104">
@@ -6509,7 +6432,7 @@
       </c>
     </row>
     <row r="22" spans="1:2" ht="15.5">
-      <c r="A22" s="159">
+      <c r="A22" s="158">
         <v>44440</v>
       </c>
       <c r="B22" s="104">
@@ -6517,7 +6440,7 @@
       </c>
     </row>
     <row r="23" spans="1:2" ht="15.5">
-      <c r="A23" s="159">
+      <c r="A23" s="158">
         <v>44470</v>
       </c>
       <c r="B23" s="104">
@@ -6525,7 +6448,7 @@
       </c>
     </row>
     <row r="24" spans="1:2" ht="15.5">
-      <c r="A24" s="159">
+      <c r="A24" s="158">
         <v>44501</v>
       </c>
       <c r="B24" s="104">
@@ -6533,7 +6456,7 @@
       </c>
     </row>
     <row r="25" spans="1:2" ht="15.5">
-      <c r="A25" s="159">
+      <c r="A25" s="158">
         <v>44531</v>
       </c>
       <c r="B25" s="105">
@@ -6541,7 +6464,7 @@
       </c>
     </row>
     <row r="26" spans="1:2" ht="15.5">
-      <c r="A26" s="159">
+      <c r="A26" s="158">
         <v>44562</v>
       </c>
       <c r="B26" s="104">
@@ -6549,7 +6472,7 @@
       </c>
     </row>
     <row r="27" spans="1:2" ht="15.5">
-      <c r="A27" s="159">
+      <c r="A27" s="158">
         <v>44593</v>
       </c>
       <c r="B27" s="104">
@@ -6557,7 +6480,7 @@
       </c>
     </row>
     <row r="28" spans="1:2" ht="15.5">
-      <c r="A28" s="159">
+      <c r="A28" s="158">
         <v>44621</v>
       </c>
       <c r="B28" s="104">
@@ -6565,7 +6488,7 @@
       </c>
     </row>
     <row r="29" spans="1:2" ht="15.5">
-      <c r="A29" s="159">
+      <c r="A29" s="158">
         <v>44652</v>
       </c>
       <c r="B29" s="104">
@@ -6573,7 +6496,7 @@
       </c>
     </row>
     <row r="30" spans="1:2" ht="15.5">
-      <c r="A30" s="159">
+      <c r="A30" s="158">
         <v>44682</v>
       </c>
       <c r="B30" s="104">
@@ -6581,7 +6504,7 @@
       </c>
     </row>
     <row r="31" spans="1:2" ht="15.5">
-      <c r="A31" s="159">
+      <c r="A31" s="158">
         <v>44713</v>
       </c>
       <c r="B31" s="104">
@@ -6589,7 +6512,7 @@
       </c>
     </row>
     <row r="32" spans="1:2" ht="15.5">
-      <c r="A32" s="159">
+      <c r="A32" s="158">
         <v>44743</v>
       </c>
       <c r="B32" s="104">
@@ -6597,7 +6520,7 @@
       </c>
     </row>
     <row r="33" spans="1:2" ht="15.5">
-      <c r="A33" s="159">
+      <c r="A33" s="158">
         <v>44774</v>
       </c>
       <c r="B33" s="104">
@@ -6605,7 +6528,7 @@
       </c>
     </row>
     <row r="34" spans="1:2" ht="15.5">
-      <c r="A34" s="159">
+      <c r="A34" s="158">
         <v>44805</v>
       </c>
       <c r="B34" s="104">
@@ -6613,7 +6536,7 @@
       </c>
     </row>
     <row r="35" spans="1:2" ht="15.5">
-      <c r="A35" s="159">
+      <c r="A35" s="158">
         <v>44835</v>
       </c>
       <c r="B35" s="104">
@@ -6621,7 +6544,7 @@
       </c>
     </row>
     <row r="36" spans="1:2" ht="15.5">
-      <c r="A36" s="159">
+      <c r="A36" s="158">
         <v>44866</v>
       </c>
       <c r="B36" s="104">
@@ -6629,10 +6552,10 @@
       </c>
     </row>
     <row r="37" spans="1:2" ht="16" thickBot="1">
-      <c r="A37" s="159">
+      <c r="A37" s="158">
         <v>44896</v>
       </c>
-      <c r="B37" s="160">
+      <c r="B37" s="159">
         <v>6504</v>
       </c>
     </row>
@@ -6671,14 +6594,14 @@
       <c r="B1" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="152" t="s">
-        <v>121</v>
+      <c r="C1" s="151" t="s">
+        <v>116</v>
       </c>
       <c r="D1" s="18" t="s">
         <v>37</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="F1" s="18" t="s">
         <v>38</v>
@@ -6703,7 +6626,7 @@
         <f>B2/$C$13</f>
         <v>0.80362385705897155</v>
       </c>
-      <c r="E2" s="153">
+      <c r="E2" s="152">
         <f>AVERAGE(D2,D14,D26)</f>
         <v>0.73392852694691335</v>
       </c>
@@ -6714,9 +6637,9 @@
       <c r="G2" s="24">
         <v>1</v>
       </c>
-      <c r="I2" s="179"/>
+      <c r="I2" s="178"/>
       <c r="J2" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="16" thickBot="1">
@@ -6731,7 +6654,7 @@
         <f t="shared" ref="D3:D13" si="0">B3/$C$13</f>
         <v>0.86704135559097395</v>
       </c>
-      <c r="E3" s="153">
+      <c r="E3" s="152">
         <f>AVERAGE(D3,D15,D27)</f>
         <v>0.82465976791108309</v>
       </c>
@@ -6755,7 +6678,7 @@
         <f>B4/$C$13</f>
         <v>0.89958896065766292</v>
       </c>
-      <c r="E4" s="153">
+      <c r="E4" s="152">
         <f t="shared" ref="E4:E13" si="2">AVERAGE(D4,D16,D28)</f>
         <v>0.84486535502079041</v>
       </c>
@@ -6766,10 +6689,10 @@
       <c r="G4" s="24">
         <v>3</v>
       </c>
-      <c r="J4" s="165" t="s">
-        <v>147</v>
-      </c>
-      <c r="K4" s="165"/>
+      <c r="J4" s="164" t="s">
+        <v>142</v>
+      </c>
+      <c r="K4" s="164"/>
     </row>
     <row r="5" spans="1:15" ht="15.5">
       <c r="A5" s="22">
@@ -6783,7 +6706,7 @@
         <f t="shared" si="0"/>
         <v>1.0072980454659843</v>
       </c>
-      <c r="E5" s="153">
+      <c r="E5" s="152">
         <f t="shared" si="2"/>
         <v>0.94253800106702668</v>
       </c>
@@ -6795,7 +6718,7 @@
         <v>4</v>
       </c>
       <c r="J5" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="K5">
         <v>0.68692857056872358</v>
@@ -6813,7 +6736,7 @@
         <f>B6/$C$13</f>
         <v>1.1653384783155776</v>
       </c>
-      <c r="E6" s="153">
+      <c r="E6" s="152">
         <f t="shared" si="2"/>
         <v>1.0824033788612222</v>
       </c>
@@ -6825,7 +6748,7 @@
         <v>5</v>
       </c>
       <c r="J6" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="K6">
         <v>0.47187086106358989</v>
@@ -6843,7 +6766,7 @@
         <f t="shared" si="0"/>
         <v>1.1267511114839359</v>
       </c>
-      <c r="E7" s="153">
+      <c r="E7" s="152">
         <f t="shared" si="2"/>
         <v>1.0760027858749039</v>
       </c>
@@ -6855,7 +6778,7 @@
         <v>6</v>
       </c>
       <c r="J7" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="K7">
         <v>0.4563376510948719</v>
@@ -6873,7 +6796,7 @@
         <f t="shared" si="0"/>
         <v>0.40298632665044881</v>
       </c>
-      <c r="E8" s="153">
+      <c r="E8" s="152">
         <f t="shared" si="2"/>
         <v>0.66488929258360752</v>
       </c>
@@ -6885,7 +6808,7 @@
         <v>7</v>
       </c>
       <c r="J8" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K8">
         <v>326.24333090974409</v>
@@ -6903,7 +6826,7 @@
         <f t="shared" si="0"/>
         <v>0.8552973743813439</v>
       </c>
-      <c r="E9" s="153">
+      <c r="E9" s="152">
         <f t="shared" si="2"/>
         <v>0.88661084214360442</v>
       </c>
@@ -6914,10 +6837,10 @@
       <c r="G9" s="24">
         <v>8</v>
       </c>
-      <c r="J9" s="163" t="s">
-        <v>152</v>
-      </c>
-      <c r="K9" s="163">
+      <c r="J9" s="162" t="s">
+        <v>147</v>
+      </c>
+      <c r="K9" s="162">
         <v>36</v>
       </c>
     </row>
@@ -6933,7 +6856,7 @@
         <f t="shared" si="0"/>
         <v>1.0106534686687358</v>
       </c>
-      <c r="E10" s="153">
+      <c r="E10" s="152">
         <f t="shared" si="2"/>
         <v>0.9400754667422464</v>
       </c>
@@ -6957,7 +6880,7 @@
         <f t="shared" si="0"/>
         <v>1.1948662024997903</v>
       </c>
-      <c r="E11" s="153">
+      <c r="E11" s="152">
         <f t="shared" si="2"/>
         <v>1.182476321568634</v>
       </c>
@@ -6969,7 +6892,7 @@
         <v>10</v>
       </c>
       <c r="J11" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="15.5">
@@ -6984,7 +6907,7 @@
         <f t="shared" si="0"/>
         <v>1.1515812431842967</v>
       </c>
-      <c r="E12" s="153">
+      <c r="E12" s="152">
         <f t="shared" si="2"/>
         <v>1.232884602717629</v>
       </c>
@@ -6995,21 +6918,21 @@
       <c r="G12" s="24">
         <v>11</v>
       </c>
-      <c r="J12" s="164"/>
-      <c r="K12" s="164" t="s">
-        <v>158</v>
-      </c>
-      <c r="L12" s="164" t="s">
-        <v>159</v>
-      </c>
-      <c r="M12" s="164" t="s">
-        <v>160</v>
-      </c>
-      <c r="N12" s="164" t="s">
-        <v>161</v>
-      </c>
-      <c r="O12" s="164" t="s">
-        <v>162</v>
+      <c r="J12" s="163"/>
+      <c r="K12" s="163" t="s">
+        <v>153</v>
+      </c>
+      <c r="L12" s="163" t="s">
+        <v>154</v>
+      </c>
+      <c r="M12" s="163" t="s">
+        <v>155</v>
+      </c>
+      <c r="N12" s="163" t="s">
+        <v>156</v>
+      </c>
+      <c r="O12" s="163" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="15.5">
@@ -7027,7 +6950,7 @@
         <f t="shared" si="0"/>
         <v>1.5149735760422782</v>
       </c>
-      <c r="E13" s="153">
+      <c r="E13" s="152">
         <f t="shared" si="2"/>
         <v>1.5886656585623395</v>
       </c>
@@ -7039,7 +6962,7 @@
         <v>12</v>
       </c>
       <c r="J13" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="K13">
         <v>1</v>
@@ -7078,7 +7001,7 @@
         <v>13</v>
       </c>
       <c r="J14" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="K14">
         <v>34</v>
@@ -7110,18 +7033,18 @@
       <c r="G15" s="24">
         <v>14</v>
       </c>
-      <c r="J15" s="163" t="s">
-        <v>156</v>
-      </c>
-      <c r="K15" s="163">
+      <c r="J15" s="162" t="s">
+        <v>151</v>
+      </c>
+      <c r="K15" s="162">
         <v>35</v>
       </c>
-      <c r="L15" s="163">
+      <c r="L15" s="162">
         <v>6852074.437764748</v>
       </c>
-      <c r="M15" s="163"/>
-      <c r="N15" s="163"/>
-      <c r="O15" s="163"/>
+      <c r="M15" s="162"/>
+      <c r="N15" s="162"/>
+      <c r="O15" s="162"/>
     </row>
     <row r="16" spans="1:15" ht="16" thickBot="1">
       <c r="A16" s="22">
@@ -7164,30 +7087,30 @@
       <c r="G17" s="24">
         <v>16</v>
       </c>
-      <c r="J17" s="164"/>
-      <c r="K17" s="164" t="s">
+      <c r="J17" s="163"/>
+      <c r="K17" s="163" t="s">
+        <v>158</v>
+      </c>
+      <c r="L17" s="163" t="s">
+        <v>146</v>
+      </c>
+      <c r="M17" s="163" t="s">
+        <v>159</v>
+      </c>
+      <c r="N17" s="163" t="s">
+        <v>160</v>
+      </c>
+      <c r="O17" s="163" t="s">
+        <v>161</v>
+      </c>
+      <c r="P17" s="163" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q17" s="163" t="s">
         <v>163</v>
       </c>
-      <c r="L17" s="164" t="s">
-        <v>151</v>
-      </c>
-      <c r="M17" s="164" t="s">
+      <c r="R17" s="163" t="s">
         <v>164</v>
-      </c>
-      <c r="N17" s="164" t="s">
-        <v>165</v>
-      </c>
-      <c r="O17" s="164" t="s">
-        <v>166</v>
-      </c>
-      <c r="P17" s="164" t="s">
-        <v>167</v>
-      </c>
-      <c r="Q17" s="164" t="s">
-        <v>168</v>
-      </c>
-      <c r="R17" s="164" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="18" spans="1:18" ht="15.5">
@@ -7211,7 +7134,7 @@
         <v>17</v>
       </c>
       <c r="J18" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="K18">
         <v>2809.0228649101136</v>
@@ -7258,31 +7181,31 @@
       <c r="G19" s="24">
         <v>18</v>
       </c>
-      <c r="J19" s="163" t="s">
+      <c r="J19" s="162" t="s">
         <v>10</v>
       </c>
-      <c r="K19" s="163">
+      <c r="K19" s="162">
         <v>28.848756924118746</v>
       </c>
-      <c r="L19" s="163">
+      <c r="L19" s="162">
         <v>5.2341495964693276</v>
       </c>
-      <c r="M19" s="163">
+      <c r="M19" s="162">
         <v>5.5116416511248643</v>
       </c>
-      <c r="N19" s="163">
+      <c r="N19" s="162">
         <v>3.715745689329591E-6</v>
       </c>
-      <c r="O19" s="163">
+      <c r="O19" s="162">
         <v>18.211685145746401</v>
       </c>
-      <c r="P19" s="163">
+      <c r="P19" s="162">
         <v>39.485828702491091</v>
       </c>
-      <c r="Q19" s="163">
+      <c r="Q19" s="162">
         <v>18.211685145746401</v>
       </c>
-      <c r="R19" s="163">
+      <c r="R19" s="162">
         <v>39.485828702491091</v>
       </c>
     </row>
@@ -7624,7 +7547,7 @@
       <c r="G35" s="24">
         <v>34</v>
       </c>
-      <c r="I35" s="154"/>
+      <c r="I35" s="153"/>
     </row>
     <row r="36" spans="1:9" ht="16" thickBot="1">
       <c r="A36" s="22">
@@ -7652,7 +7575,7 @@
       <c r="A37" s="22">
         <v>44896</v>
       </c>
-      <c r="B37" s="160">
+      <c r="B37" s="159">
         <v>6504</v>
       </c>
       <c r="C37" s="134">
@@ -7675,240 +7598,240 @@
         <v>40</v>
       </c>
       <c r="I37" s="85" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="38" spans="1:9">
       <c r="A38" s="133"/>
-      <c r="B38" s="155"/>
-      <c r="C38" s="156"/>
-      <c r="D38" s="156"/>
-      <c r="E38" s="157"/>
-      <c r="F38" s="158"/>
+      <c r="B38" s="154"/>
+      <c r="C38" s="155"/>
+      <c r="D38" s="155"/>
+      <c r="E38" s="156"/>
+      <c r="F38" s="157"/>
       <c r="G38" s="24">
         <v>37</v>
       </c>
       <c r="H38" s="84">
-        <f>$K$19*G38+$K$18</f>
+        <f t="shared" ref="H38:H49" si="7">$K$19*G38+$K$18</f>
         <v>3876.426871102507</v>
       </c>
       <c r="I38" s="84">
-        <f>H38*E2</f>
+        <f t="shared" ref="I38:I49" si="8">H38*E2</f>
         <v>2845.0202633256954</v>
       </c>
     </row>
     <row r="39" spans="1:9">
       <c r="A39" s="138"/>
-      <c r="B39" s="184"/>
-      <c r="C39" s="179"/>
-      <c r="D39" s="179"/>
-      <c r="E39" s="185"/>
-      <c r="F39" s="186"/>
+      <c r="B39" s="179"/>
+      <c r="C39" s="178"/>
+      <c r="D39" s="178"/>
+      <c r="E39" s="180"/>
+      <c r="F39" s="181"/>
       <c r="G39" s="24">
         <v>38</v>
       </c>
       <c r="H39" s="84">
-        <f>$K$19*G39+$K$18</f>
+        <f t="shared" si="7"/>
         <v>3905.2756280266258</v>
       </c>
       <c r="I39" s="84">
-        <f>H39*E3</f>
+        <f t="shared" si="8"/>
         <v>3220.5236930372466</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40" s="138"/>
-      <c r="B40" s="184"/>
-      <c r="C40" s="179"/>
-      <c r="D40" s="179"/>
-      <c r="E40" s="185"/>
-      <c r="F40" s="186"/>
+      <c r="B40" s="179"/>
+      <c r="C40" s="178"/>
+      <c r="D40" s="178"/>
+      <c r="E40" s="180"/>
+      <c r="F40" s="181"/>
       <c r="G40" s="24">
         <v>39</v>
       </c>
       <c r="H40" s="84">
-        <f>$K$19*G40+$K$18</f>
+        <f t="shared" si="7"/>
         <v>3934.1243849507446</v>
       </c>
       <c r="I40" s="84">
-        <f>H40*E4</f>
+        <f t="shared" si="8"/>
         <v>3323.8053951873594</v>
       </c>
     </row>
     <row r="41" spans="1:9">
       <c r="A41" s="138"/>
-      <c r="B41" s="184"/>
-      <c r="C41" s="179"/>
-      <c r="D41" s="179"/>
-      <c r="E41" s="185"/>
-      <c r="F41" s="186"/>
+      <c r="B41" s="179"/>
+      <c r="C41" s="178"/>
+      <c r="D41" s="178"/>
+      <c r="E41" s="180"/>
+      <c r="F41" s="181"/>
       <c r="G41" s="24">
         <v>40</v>
       </c>
       <c r="H41" s="84">
-        <f>$K$19*G41+$K$18</f>
+        <f t="shared" si="7"/>
         <v>3962.9731418748634</v>
       </c>
       <c r="I41" s="84">
-        <f>H41*E5</f>
+        <f t="shared" si="8"/>
         <v>3735.2527834250482</v>
       </c>
     </row>
     <row r="42" spans="1:9">
       <c r="A42" s="138"/>
-      <c r="B42" s="184"/>
-      <c r="C42" s="179"/>
-      <c r="D42" s="179"/>
-      <c r="E42" s="185"/>
-      <c r="F42" s="186"/>
+      <c r="B42" s="179"/>
+      <c r="C42" s="178"/>
+      <c r="D42" s="178"/>
+      <c r="E42" s="180"/>
+      <c r="F42" s="181"/>
       <c r="G42" s="24">
         <v>41</v>
       </c>
       <c r="H42" s="84">
-        <f>$K$19*G42+$K$18</f>
+        <f t="shared" si="7"/>
         <v>3991.8218987989821</v>
       </c>
       <c r="I42" s="84">
-        <f>H42*E6</f>
+        <f t="shared" si="8"/>
         <v>4320.7615110722381</v>
       </c>
     </row>
     <row r="43" spans="1:9">
       <c r="A43" s="138"/>
-      <c r="B43" s="184"/>
-      <c r="C43" s="179"/>
-      <c r="D43" s="179"/>
-      <c r="E43" s="185"/>
-      <c r="F43" s="186"/>
+      <c r="B43" s="179"/>
+      <c r="C43" s="178"/>
+      <c r="D43" s="178"/>
+      <c r="E43" s="180"/>
+      <c r="F43" s="181"/>
       <c r="G43" s="24">
         <v>42</v>
       </c>
       <c r="H43" s="84">
-        <f>$K$19*G43+$K$18</f>
+        <f t="shared" si="7"/>
         <v>4020.6706557231009</v>
       </c>
       <c r="I43" s="84">
-        <f>H43*E7</f>
+        <f t="shared" si="8"/>
         <v>4326.2528266435338</v>
       </c>
     </row>
     <row r="44" spans="1:9">
       <c r="A44" s="138"/>
-      <c r="B44" s="184"/>
-      <c r="C44" s="179"/>
-      <c r="D44" s="179"/>
-      <c r="E44" s="185"/>
-      <c r="F44" s="186"/>
+      <c r="B44" s="179"/>
+      <c r="C44" s="178"/>
+      <c r="D44" s="178"/>
+      <c r="E44" s="180"/>
+      <c r="F44" s="181"/>
       <c r="G44" s="24">
         <v>43</v>
       </c>
       <c r="H44" s="84">
-        <f>$K$19*G44+$K$18</f>
+        <f t="shared" si="7"/>
         <v>4049.5194126472197</v>
       </c>
       <c r="I44" s="84">
-        <f>H44*E8</f>
+        <f t="shared" si="8"/>
         <v>2692.4820975785956</v>
       </c>
     </row>
     <row r="45" spans="1:9">
       <c r="A45" s="138"/>
-      <c r="B45" s="184"/>
-      <c r="C45" s="179"/>
-      <c r="D45" s="179"/>
-      <c r="E45" s="185"/>
-      <c r="F45" s="186"/>
+      <c r="B45" s="179"/>
+      <c r="C45" s="178"/>
+      <c r="D45" s="178"/>
+      <c r="E45" s="180"/>
+      <c r="F45" s="181"/>
       <c r="G45" s="24">
         <v>44</v>
       </c>
       <c r="H45" s="84">
-        <f>$K$19*G45+$K$18</f>
+        <f t="shared" si="7"/>
         <v>4078.3681695713385</v>
       </c>
       <c r="I45" s="84">
-        <f>H45*E9</f>
+        <f t="shared" si="8"/>
         <v>3615.9254373953149</v>
       </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" s="138"/>
-      <c r="B46" s="184"/>
-      <c r="C46" s="179"/>
-      <c r="D46" s="179"/>
-      <c r="E46" s="185"/>
-      <c r="F46" s="186"/>
+      <c r="B46" s="179"/>
+      <c r="C46" s="178"/>
+      <c r="D46" s="178"/>
+      <c r="E46" s="180"/>
+      <c r="F46" s="181"/>
       <c r="G46" s="24">
         <v>45</v>
       </c>
       <c r="H46" s="84">
-        <f>$K$19*G46+$K$18</f>
+        <f t="shared" si="7"/>
         <v>4107.2169264954573</v>
       </c>
       <c r="I46" s="84">
-        <f>H46*E10</f>
+        <f t="shared" si="8"/>
         <v>3861.0938691868719</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" s="138"/>
-      <c r="B47" s="184"/>
-      <c r="C47" s="179"/>
-      <c r="D47" s="179"/>
-      <c r="E47" s="185"/>
-      <c r="F47" s="186"/>
+      <c r="B47" s="179"/>
+      <c r="C47" s="178"/>
+      <c r="D47" s="178"/>
+      <c r="E47" s="180"/>
+      <c r="F47" s="181"/>
       <c r="G47" s="24">
         <v>46</v>
       </c>
       <c r="H47" s="84">
-        <f>$K$19*G47+$K$18</f>
+        <f t="shared" si="7"/>
         <v>4136.0656834195761</v>
       </c>
       <c r="I47" s="84">
-        <f>H47*E11</f>
+        <f t="shared" si="8"/>
         <v>4890.7997350962387</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" s="138"/>
-      <c r="B48" s="184"/>
-      <c r="C48" s="179"/>
-      <c r="D48" s="179"/>
-      <c r="E48" s="185"/>
-      <c r="F48" s="186"/>
+      <c r="B48" s="179"/>
+      <c r="C48" s="178"/>
+      <c r="D48" s="178"/>
+      <c r="E48" s="180"/>
+      <c r="F48" s="181"/>
       <c r="G48" s="24">
         <v>47</v>
       </c>
       <c r="H48" s="84">
-        <f>$K$19*G48+$K$18</f>
+        <f t="shared" si="7"/>
         <v>4164.9144403436949</v>
       </c>
       <c r="I48" s="84">
-        <f>H48*E12</f>
+        <f t="shared" si="8"/>
         <v>5134.8588851360528</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="15" thickBot="1">
       <c r="A49" s="138"/>
-      <c r="B49" s="187"/>
-      <c r="C49" s="188"/>
-      <c r="D49" s="188"/>
-      <c r="E49" s="189"/>
-      <c r="F49" s="190"/>
+      <c r="B49" s="182"/>
+      <c r="C49" s="183"/>
+      <c r="D49" s="183"/>
+      <c r="E49" s="184"/>
+      <c r="F49" s="185"/>
       <c r="G49" s="24">
         <v>48</v>
       </c>
       <c r="H49" s="84">
-        <f>$K$19*G49+$K$18</f>
+        <f t="shared" si="7"/>
         <v>4193.7631972678137</v>
       </c>
       <c r="I49" s="84">
-        <f>H49*E13</f>
+        <f t="shared" si="8"/>
         <v>6662.4875716419738</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="47" thickBot="1">
       <c r="C50" s="135" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E50" s="136" t="s">
         <v>98</v>
@@ -7917,7 +7840,7 @@
         <v>96</v>
       </c>
       <c r="H50" s="112" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="I50" s="86">
         <f>AVERAGE(I38:I49)</f>
@@ -7937,8 +7860,8 @@
         <f>SUM(F2:F37)</f>
         <v>120338.09524822717</v>
       </c>
-      <c r="H51" s="183"/>
-      <c r="I51" s="183"/>
+      <c r="H51" s="186"/>
+      <c r="I51" s="186"/>
     </row>
     <row r="52" spans="1:9" ht="47" thickBot="1">
       <c r="C52" s="55" t="s">
@@ -7947,8 +7870,8 @@
       <c r="F52" s="88" t="s">
         <v>97</v>
       </c>
-      <c r="H52" s="183"/>
-      <c r="I52" s="183"/>
+      <c r="H52" s="186"/>
+      <c r="I52" s="186"/>
     </row>
     <row r="53" spans="1:9" ht="15" thickBot="1">
       <c r="C53" s="63">
@@ -8007,9 +7930,9 @@
       <c r="A1" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="191"/>
-      <c r="C1" s="191"/>
-      <c r="D1" s="192"/>
+      <c r="B1" s="187"/>
+      <c r="C1" s="187"/>
+      <c r="D1" s="188"/>
       <c r="E1" s="27" t="s">
         <v>29</v>
       </c>
@@ -8020,15 +7943,15 @@
         <v>31</v>
       </c>
       <c r="Z1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:26">
       <c r="A2" s="52"/>
-      <c r="B2" s="191"/>
-      <c r="C2" s="191"/>
-      <c r="D2" s="192"/>
-      <c r="E2" s="166">
+      <c r="B2" s="187"/>
+      <c r="C2" s="187"/>
+      <c r="D2" s="188"/>
+      <c r="E2" s="165">
         <v>4000</v>
       </c>
       <c r="F2" s="27">
@@ -9070,23 +8993,23 @@
     </row>
     <row r="27" spans="1:16">
       <c r="A27" s="52"/>
-      <c r="B27" s="179"/>
-      <c r="C27" s="179"/>
-      <c r="D27" s="179"/>
-      <c r="E27" s="179"/>
-      <c r="F27" s="179"/>
-      <c r="G27" s="179"/>
+      <c r="B27" s="178"/>
+      <c r="C27" s="178"/>
+      <c r="D27" s="178"/>
+      <c r="E27" s="178"/>
+      <c r="F27" s="178"/>
+      <c r="G27" s="178"/>
     </row>
     <row r="28" spans="1:16" ht="15" thickBot="1">
       <c r="A28" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="B28" s="179"/>
-      <c r="C28" s="179"/>
-      <c r="D28" s="179"/>
-      <c r="E28" s="179"/>
-      <c r="F28" s="179"/>
-      <c r="G28" s="179"/>
+      <c r="B28" s="178"/>
+      <c r="C28" s="178"/>
+      <c r="D28" s="178"/>
+      <c r="E28" s="178"/>
+      <c r="F28" s="178"/>
+      <c r="G28" s="178"/>
     </row>
     <row r="29" spans="1:16">
       <c r="A29" s="58" t="s">
@@ -11192,9 +11115,9 @@
       <c r="A1" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="191"/>
-      <c r="C1" s="191"/>
-      <c r="D1" s="192"/>
+      <c r="B1" s="187"/>
+      <c r="C1" s="187"/>
+      <c r="D1" s="188"/>
       <c r="E1" s="27" t="s">
         <v>29</v>
       </c>
@@ -11207,10 +11130,10 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="52"/>
-      <c r="B2" s="191"/>
-      <c r="C2" s="191"/>
-      <c r="D2" s="192"/>
-      <c r="E2" s="167">
+      <c r="B2" s="187"/>
+      <c r="C2" s="187"/>
+      <c r="D2" s="188"/>
+      <c r="E2" s="166">
         <f>4000*1.32</f>
         <v>5280</v>
       </c>
@@ -14415,25 +14338,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16" customHeight="1">
-      <c r="A1" s="193"/>
+      <c r="A1" s="192"/>
       <c r="B1" s="20" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16" customHeight="1" thickBot="1">
-      <c r="A2" s="193"/>
+      <c r="A2" s="192"/>
     </row>
     <row r="3" spans="1:5" ht="19.5" customHeight="1" thickBot="1">
-      <c r="A3" s="193"/>
+      <c r="A3" s="192"/>
       <c r="B3" s="33"/>
-      <c r="C3" s="180" t="s">
+      <c r="C3" s="189" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="181"/>
-      <c r="E3" s="182"/>
+      <c r="D3" s="190"/>
+      <c r="E3" s="191"/>
     </row>
     <row r="4" spans="1:5" ht="18.5" customHeight="1" thickBot="1">
-      <c r="A4" s="193"/>
+      <c r="A4" s="192"/>
       <c r="B4" s="34" t="s">
         <v>65</v>
       </c>
@@ -14448,7 +14371,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.5" thickTop="1" thickBot="1">
-      <c r="A5" s="193"/>
+      <c r="A5" s="192"/>
       <c r="B5" s="94" t="s">
         <v>41</v>
       </c>
@@ -14463,7 +14386,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="15.5" thickTop="1" thickBot="1">
-      <c r="A6" s="193"/>
+      <c r="A6" s="192"/>
       <c r="B6" s="95" t="s">
         <v>87</v>
       </c>
@@ -14503,11 +14426,11 @@
     </row>
     <row r="11" spans="1:5" ht="15" thickBot="1">
       <c r="B11" s="33"/>
-      <c r="C11" s="180" t="s">
+      <c r="C11" s="189" t="s">
         <v>64</v>
       </c>
-      <c r="D11" s="181"/>
-      <c r="E11" s="182"/>
+      <c r="D11" s="190"/>
+      <c r="E11" s="191"/>
     </row>
     <row r="12" spans="1:5" ht="15" thickBot="1">
       <c r="B12" s="34" t="s">
@@ -14581,11 +14504,11 @@
     </row>
     <row r="18" spans="2:5" ht="15" thickBot="1">
       <c r="B18" s="33"/>
-      <c r="C18" s="180" t="s">
+      <c r="C18" s="189" t="s">
         <v>64</v>
       </c>
-      <c r="D18" s="181"/>
-      <c r="E18" s="182"/>
+      <c r="D18" s="190"/>
+      <c r="E18" s="191"/>
     </row>
     <row r="19" spans="2:5" ht="15" thickBot="1">
       <c r="B19" s="34" t="s">
@@ -14659,11 +14582,11 @@
     </row>
     <row r="25" spans="2:5" ht="15" thickBot="1">
       <c r="B25" s="33"/>
-      <c r="C25" s="180" t="s">
+      <c r="C25" s="189" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="181"/>
-      <c r="E25" s="182"/>
+      <c r="D25" s="190"/>
+      <c r="E25" s="191"/>
     </row>
     <row r="26" spans="2:5" ht="15" thickBot="1">
       <c r="B26" s="34" t="s">
@@ -14739,11 +14662,11 @@
       <c r="B32" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="C32" s="180" t="s">
+      <c r="C32" s="189" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="181"/>
-      <c r="E32" s="182"/>
+      <c r="D32" s="190"/>
+      <c r="E32" s="191"/>
     </row>
     <row r="33" spans="2:5" ht="15" thickBot="1">
       <c r="B33" s="34" t="s">
@@ -15080,36 +15003,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="112" customFormat="1" ht="29.5" thickBot="1">
-      <c r="A1" s="178" t="s">
+      <c r="A1" s="177" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="177" t="s">
+      <c r="B1" s="176" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="176" t="s">
-        <v>172</v>
-      </c>
-      <c r="D1" s="176" t="s">
-        <v>171</v>
-      </c>
-      <c r="E1" s="176" t="s">
-        <v>170</v>
+      <c r="C1" s="175" t="s">
+        <v>167</v>
+      </c>
+      <c r="D1" s="175" t="s">
+        <v>166</v>
+      </c>
+      <c r="E1" s="175" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="15.5">
       <c r="A2" s="22">
         <v>44470</v>
       </c>
-      <c r="B2" s="173">
+      <c r="B2" s="172">
         <v>3634</v>
       </c>
-      <c r="C2" s="172">
+      <c r="C2" s="171">
         <v>30</v>
       </c>
-      <c r="D2" s="172">
+      <c r="D2" s="171">
         <v>1</v>
       </c>
-      <c r="E2" s="172">
+      <c r="E2" s="171">
         <v>0</v>
       </c>
     </row>
@@ -15117,16 +15040,16 @@
       <c r="A3" s="22">
         <v>44501</v>
       </c>
-      <c r="B3" s="173">
+      <c r="B3" s="172">
         <v>4550</v>
       </c>
-      <c r="C3" s="172">
+      <c r="C3" s="171">
         <v>40</v>
       </c>
-      <c r="D3" s="172">
-        <v>0</v>
-      </c>
-      <c r="E3" s="172">
+      <c r="D3" s="171">
+        <v>0</v>
+      </c>
+      <c r="E3" s="171">
         <v>1</v>
       </c>
     </row>
@@ -15134,34 +15057,34 @@
       <c r="A4" s="22">
         <v>44531</v>
       </c>
-      <c r="B4" s="175">
+      <c r="B4" s="174">
         <v>5330</v>
       </c>
-      <c r="C4" s="172">
+      <c r="C4" s="171">
         <v>55</v>
       </c>
-      <c r="D4" s="172">
+      <c r="D4" s="171">
         <v>1</v>
       </c>
-      <c r="E4" s="172">
-        <v>0</v>
-      </c>
-      <c r="H4" s="174"/>
+      <c r="E4" s="171">
+        <v>0</v>
+      </c>
+      <c r="H4" s="173"/>
     </row>
     <row r="5" spans="1:25" ht="15.5">
       <c r="A5" s="22">
         <v>44562</v>
       </c>
-      <c r="B5" s="173">
+      <c r="B5" s="172">
         <v>3100</v>
       </c>
-      <c r="C5" s="172">
+      <c r="C5" s="171">
         <v>30</v>
       </c>
-      <c r="D5" s="172">
-        <v>0</v>
-      </c>
-      <c r="E5" s="172">
+      <c r="D5" s="171">
+        <v>0</v>
+      </c>
+      <c r="E5" s="171">
         <v>1</v>
       </c>
     </row>
@@ -15169,16 +15092,16 @@
       <c r="A6" s="22">
         <v>44593</v>
       </c>
-      <c r="B6" s="173">
+      <c r="B6" s="172">
         <v>2999</v>
       </c>
-      <c r="C6" s="172">
+      <c r="C6" s="171">
         <v>30</v>
       </c>
-      <c r="D6" s="172">
-        <v>0</v>
-      </c>
-      <c r="E6" s="172">
+      <c r="D6" s="171">
+        <v>0</v>
+      </c>
+      <c r="E6" s="171">
         <v>1</v>
       </c>
     </row>
@@ -15186,16 +15109,16 @@
       <c r="A7" s="22">
         <v>44621</v>
       </c>
-      <c r="B7" s="173">
+      <c r="B7" s="172">
         <v>3051</v>
       </c>
-      <c r="C7" s="172">
+      <c r="C7" s="171">
         <v>35</v>
       </c>
-      <c r="D7" s="172">
+      <c r="D7" s="171">
         <v>1</v>
       </c>
-      <c r="E7" s="172">
+      <c r="E7" s="171">
         <v>0</v>
       </c>
     </row>
@@ -15203,16 +15126,16 @@
       <c r="A8" s="22">
         <v>44652</v>
       </c>
-      <c r="B8" s="173">
+      <c r="B8" s="172">
         <v>3753</v>
       </c>
-      <c r="C8" s="172">
+      <c r="C8" s="171">
         <v>35</v>
       </c>
-      <c r="D8" s="172">
-        <v>0</v>
-      </c>
-      <c r="E8" s="172">
+      <c r="D8" s="171">
+        <v>0</v>
+      </c>
+      <c r="E8" s="171">
         <v>1</v>
       </c>
     </row>
@@ -15220,16 +15143,16 @@
       <c r="A9" s="22">
         <v>44682</v>
       </c>
-      <c r="B9" s="173">
+      <c r="B9" s="172">
         <v>3709</v>
       </c>
-      <c r="C9" s="172">
+      <c r="C9" s="171">
         <v>35</v>
       </c>
-      <c r="D9" s="172">
-        <v>0</v>
-      </c>
-      <c r="E9" s="172">
+      <c r="D9" s="171">
+        <v>0</v>
+      </c>
+      <c r="E9" s="171">
         <v>1</v>
       </c>
     </row>
@@ -15237,16 +15160,16 @@
       <c r="A10" s="22">
         <v>44713</v>
       </c>
-      <c r="B10" s="173">
+      <c r="B10" s="172">
         <v>3930</v>
       </c>
-      <c r="C10" s="172">
+      <c r="C10" s="171">
         <v>40</v>
       </c>
-      <c r="D10" s="172">
+      <c r="D10" s="171">
         <v>1</v>
       </c>
-      <c r="E10" s="172">
+      <c r="E10" s="171">
         <v>0</v>
       </c>
     </row>
@@ -15254,16 +15177,16 @@
       <c r="A11" s="22">
         <v>44743</v>
       </c>
-      <c r="B11" s="173">
+      <c r="B11" s="172">
         <v>2949</v>
       </c>
-      <c r="C11" s="172">
+      <c r="C11" s="171">
         <v>40</v>
       </c>
-      <c r="D11" s="172">
-        <v>0</v>
-      </c>
-      <c r="E11" s="172">
+      <c r="D11" s="171">
+        <v>0</v>
+      </c>
+      <c r="E11" s="171">
         <v>1</v>
       </c>
     </row>
@@ -15271,62 +15194,62 @@
       <c r="A12" s="22">
         <v>44774</v>
       </c>
-      <c r="B12" s="173">
+      <c r="B12" s="172">
         <v>3348</v>
       </c>
-      <c r="C12" s="172">
+      <c r="C12" s="171">
         <v>45</v>
       </c>
-      <c r="D12" s="172">
-        <v>0</v>
-      </c>
-      <c r="E12" s="172">
+      <c r="D12" s="171">
+        <v>0</v>
+      </c>
+      <c r="E12" s="171">
         <v>1</v>
       </c>
-      <c r="T12" s="171"/>
-      <c r="U12" s="171"/>
-      <c r="V12" s="171"/>
-      <c r="W12" s="171"/>
-      <c r="X12" s="171"/>
-      <c r="Y12" s="171"/>
+      <c r="T12" s="170"/>
+      <c r="U12" s="170"/>
+      <c r="V12" s="170"/>
+      <c r="W12" s="170"/>
+      <c r="X12" s="170"/>
+      <c r="Y12" s="170"/>
     </row>
     <row r="13" spans="1:25" ht="15.5">
       <c r="A13" s="22">
         <v>44805</v>
       </c>
-      <c r="B13" s="173">
+      <c r="B13" s="172">
         <v>3400</v>
       </c>
-      <c r="C13" s="172">
+      <c r="C13" s="171">
         <v>40</v>
       </c>
-      <c r="D13" s="172">
-        <v>0</v>
-      </c>
-      <c r="E13" s="172">
+      <c r="D13" s="171">
+        <v>0</v>
+      </c>
+      <c r="E13" s="171">
         <v>1</v>
       </c>
-      <c r="J13" s="171"/>
-      <c r="K13" s="171"/>
-      <c r="L13" s="171"/>
-      <c r="M13" s="171"/>
-      <c r="N13" s="171"/>
-      <c r="O13" s="171"/>
+      <c r="J13" s="170"/>
+      <c r="K13" s="170"/>
+      <c r="L13" s="170"/>
+      <c r="M13" s="170"/>
+      <c r="N13" s="170"/>
+      <c r="O13" s="170"/>
     </row>
     <row r="14" spans="1:25" ht="15.5">
       <c r="A14" s="22">
         <v>44835</v>
       </c>
-      <c r="B14" s="173">
+      <c r="B14" s="172">
         <v>4400</v>
       </c>
-      <c r="C14" s="172">
+      <c r="C14" s="171">
         <v>55</v>
       </c>
-      <c r="D14" s="172">
+      <c r="D14" s="171">
         <v>1</v>
       </c>
-      <c r="E14" s="172">
+      <c r="E14" s="171">
         <v>0</v>
       </c>
     </row>
@@ -15334,16 +15257,16 @@
       <c r="A15" s="22">
         <v>44866</v>
       </c>
-      <c r="B15" s="173">
+      <c r="B15" s="172">
         <v>5079</v>
       </c>
-      <c r="C15" s="172">
+      <c r="C15" s="171">
         <v>55</v>
       </c>
-      <c r="D15" s="172">
+      <c r="D15" s="171">
         <v>1</v>
       </c>
-      <c r="E15" s="172">
+      <c r="E15" s="171">
         <v>0</v>
       </c>
     </row>
@@ -15351,16 +15274,16 @@
       <c r="A16" s="22">
         <v>44896</v>
       </c>
-      <c r="B16" s="173">
+      <c r="B16" s="172">
         <v>6087</v>
       </c>
-      <c r="C16" s="172">
+      <c r="C16" s="171">
         <v>60</v>
       </c>
-      <c r="D16" s="172">
+      <c r="D16" s="171">
         <v>1</v>
       </c>
-      <c r="E16" s="172">
+      <c r="E16" s="171">
         <v>0</v>
       </c>
     </row>
@@ -15372,18 +15295,18 @@
         <f>$I$38+($I$39*C17)+($I$40*D17)</f>
         <v>1949.7956204379564</v>
       </c>
-      <c r="C17" s="170">
+      <c r="C17" s="169">
         <v>15</v>
       </c>
-      <c r="D17" s="170">
-        <v>0</v>
-      </c>
-      <c r="E17" s="170">
+      <c r="D17" s="169">
+        <v>0</v>
+      </c>
+      <c r="E17" s="169">
         <v>1</v>
       </c>
-      <c r="K17" s="171"/>
-      <c r="L17" s="171"/>
-      <c r="M17" s="171"/>
+      <c r="K17" s="170"/>
+      <c r="L17" s="170"/>
+      <c r="M17" s="170"/>
     </row>
     <row r="18" spans="1:13">
       <c r="A18" s="22">
@@ -15393,16 +15316,16 @@
         <f t="shared" ref="B18:B28" si="0">$I$38+($I$39*C18)+($I$40*D18)</f>
         <v>2298.6423357664235</v>
       </c>
-      <c r="C18" s="170">
+      <c r="C18" s="169">
         <v>20</v>
       </c>
-      <c r="D18" s="170">
-        <v>0</v>
-      </c>
-      <c r="E18" s="170">
+      <c r="D18" s="169">
+        <v>0</v>
+      </c>
+      <c r="E18" s="169">
         <v>1</v>
       </c>
-      <c r="J18" s="171"/>
+      <c r="J18" s="170"/>
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="22">
@@ -15412,13 +15335,13 @@
         <f t="shared" si="0"/>
         <v>2298.6423357664235</v>
       </c>
-      <c r="C19" s="170">
+      <c r="C19" s="169">
         <v>20</v>
       </c>
-      <c r="D19" s="170">
-        <v>0</v>
-      </c>
-      <c r="E19" s="170">
+      <c r="D19" s="169">
+        <v>0</v>
+      </c>
+      <c r="E19" s="169">
         <v>1</v>
       </c>
     </row>
@@ -15430,13 +15353,13 @@
         <f t="shared" si="0"/>
         <v>2647.4890510948908</v>
       </c>
-      <c r="C20" s="170">
+      <c r="C20" s="169">
         <v>25</v>
       </c>
-      <c r="D20" s="170">
-        <v>0</v>
-      </c>
-      <c r="E20" s="170">
+      <c r="D20" s="169">
+        <v>0</v>
+      </c>
+      <c r="E20" s="169">
         <v>1</v>
       </c>
     </row>
@@ -15448,13 +15371,13 @@
         <f t="shared" si="0"/>
         <v>2647.4890510948908</v>
       </c>
-      <c r="C21" s="170">
+      <c r="C21" s="169">
         <v>25</v>
       </c>
-      <c r="D21" s="170">
-        <v>0</v>
-      </c>
-      <c r="E21" s="170">
+      <c r="D21" s="169">
+        <v>0</v>
+      </c>
+      <c r="E21" s="169">
         <v>1</v>
       </c>
     </row>
@@ -15466,17 +15389,17 @@
         <f t="shared" si="0"/>
         <v>3654.3722627737229</v>
       </c>
-      <c r="C22" s="170">
+      <c r="C22" s="169">
         <v>35</v>
       </c>
-      <c r="D22" s="170">
+      <c r="D22" s="169">
         <v>1</v>
       </c>
-      <c r="E22" s="170">
+      <c r="E22" s="169">
         <v>0</v>
       </c>
       <c r="H22" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="15" thickBot="1">
@@ -15487,13 +15410,13 @@
         <f t="shared" si="0"/>
         <v>3654.3722627737229</v>
       </c>
-      <c r="C23" s="170">
+      <c r="C23" s="169">
         <v>35</v>
       </c>
-      <c r="D23" s="170">
+      <c r="D23" s="169">
         <v>1</v>
       </c>
-      <c r="E23" s="170">
+      <c r="E23" s="169">
         <v>0</v>
       </c>
     </row>
@@ -15505,19 +15428,19 @@
         <f>$I$38+($I$39*C24)+($I$40*D24)</f>
         <v>2647.4890510948908</v>
       </c>
-      <c r="C24" s="170">
+      <c r="C24" s="169">
         <v>25</v>
       </c>
-      <c r="D24" s="170">
-        <v>0</v>
-      </c>
-      <c r="E24" s="170">
+      <c r="D24" s="169">
+        <v>0</v>
+      </c>
+      <c r="E24" s="169">
         <v>1</v>
       </c>
-      <c r="H24" s="165" t="s">
-        <v>147</v>
-      </c>
-      <c r="I24" s="165"/>
+      <c r="H24" s="164" t="s">
+        <v>142</v>
+      </c>
+      <c r="I24" s="164"/>
     </row>
     <row r="25" spans="1:13">
       <c r="A25" s="22">
@@ -15527,17 +15450,17 @@
         <f t="shared" si="0"/>
         <v>2996.3357664233581</v>
       </c>
-      <c r="C25" s="170">
+      <c r="C25" s="169">
         <v>30</v>
       </c>
-      <c r="D25" s="170">
-        <v>0</v>
-      </c>
-      <c r="E25" s="170">
+      <c r="D25" s="169">
+        <v>0</v>
+      </c>
+      <c r="E25" s="169">
         <v>1</v>
       </c>
       <c r="H25" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="I25">
         <v>0.84434540565369609</v>
@@ -15551,17 +15474,17 @@
         <f t="shared" si="0"/>
         <v>4003.2189781021893</v>
       </c>
-      <c r="C26" s="170">
+      <c r="C26" s="169">
         <v>40</v>
       </c>
-      <c r="D26" s="170">
+      <c r="D26" s="169">
         <v>1</v>
       </c>
-      <c r="E26" s="170">
+      <c r="E26" s="169">
         <v>0</v>
       </c>
       <c r="H26" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="I26">
         <v>0.71291916404850464</v>
@@ -15575,17 +15498,17 @@
         <f t="shared" si="0"/>
         <v>4003.2189781021893</v>
       </c>
-      <c r="C27" s="170">
+      <c r="C27" s="169">
         <v>40</v>
       </c>
-      <c r="D27" s="170">
+      <c r="D27" s="169">
         <v>1</v>
       </c>
-      <c r="E27" s="170">
+      <c r="E27" s="169">
         <v>0</v>
       </c>
       <c r="H27" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="I27">
         <v>0.66507235805658871</v>
@@ -15599,67 +15522,67 @@
         <f t="shared" si="0"/>
         <v>4352.0656934306571</v>
       </c>
-      <c r="C28" s="170">
+      <c r="C28" s="169">
         <v>45</v>
       </c>
-      <c r="D28" s="170">
+      <c r="D28" s="169">
         <v>1</v>
       </c>
-      <c r="E28" s="170">
+      <c r="E28" s="169">
         <v>0</v>
       </c>
       <c r="H28" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="I28">
         <v>549.18651186779721</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="16" thickBot="1">
-      <c r="A29" s="169"/>
-      <c r="H29" s="163" t="s">
-        <v>152</v>
-      </c>
-      <c r="I29" s="163">
+      <c r="A29" s="168"/>
+      <c r="H29" s="162" t="s">
+        <v>147</v>
+      </c>
+      <c r="I29" s="162">
         <v>15</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="15.5">
-      <c r="A30" s="169"/>
+      <c r="A30" s="168"/>
     </row>
     <row r="31" spans="1:13" ht="16" thickBot="1">
-      <c r="A31" s="169"/>
+      <c r="A31" s="168"/>
       <c r="H31" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="15.5">
-      <c r="A32" s="169"/>
+      <c r="A32" s="168"/>
       <c r="B32">
         <f>SUM(B17:B28)</f>
         <v>37153.131386861307</v>
       </c>
-      <c r="H32" s="164"/>
-      <c r="I32" s="164" t="s">
-        <v>158</v>
-      </c>
-      <c r="J32" s="164" t="s">
-        <v>159</v>
-      </c>
-      <c r="K32" s="164" t="s">
-        <v>160</v>
-      </c>
-      <c r="L32" s="164" t="s">
-        <v>161</v>
-      </c>
-      <c r="M32" s="164" t="s">
-        <v>162</v>
+      <c r="H32" s="163"/>
+      <c r="I32" s="163" t="s">
+        <v>153</v>
+      </c>
+      <c r="J32" s="163" t="s">
+        <v>154</v>
+      </c>
+      <c r="K32" s="163" t="s">
+        <v>155</v>
+      </c>
+      <c r="L32" s="163" t="s">
+        <v>156</v>
+      </c>
+      <c r="M32" s="163" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="33" spans="1:16" ht="15.5">
-      <c r="A33" s="169"/>
+      <c r="A33" s="168"/>
       <c r="H33" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="I33">
         <v>2</v>
@@ -15678,9 +15601,9 @@
       </c>
     </row>
     <row r="34" spans="1:16" ht="15.5">
-      <c r="A34" s="169"/>
+      <c r="A34" s="168"/>
       <c r="H34" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="I34">
         <v>12</v>
@@ -15693,55 +15616,55 @@
       </c>
     </row>
     <row r="35" spans="1:16" ht="16" thickBot="1">
-      <c r="A35" s="169"/>
-      <c r="H35" s="163" t="s">
-        <v>156</v>
-      </c>
-      <c r="I35" s="163">
+      <c r="A35" s="168"/>
+      <c r="H35" s="162" t="s">
+        <v>151</v>
+      </c>
+      <c r="I35" s="162">
         <v>14</v>
       </c>
-      <c r="J35" s="163">
+      <c r="J35" s="162">
         <v>12607145.600000001</v>
       </c>
-      <c r="K35" s="163"/>
-      <c r="L35" s="163"/>
-      <c r="M35" s="163"/>
+      <c r="K35" s="162"/>
+      <c r="L35" s="162"/>
+      <c r="M35" s="162"/>
     </row>
     <row r="36" spans="1:16" ht="16" thickBot="1">
-      <c r="A36" s="169"/>
+      <c r="A36" s="168"/>
     </row>
     <row r="37" spans="1:16" ht="15.5">
-      <c r="A37" s="169"/>
-      <c r="H37" s="164"/>
-      <c r="I37" s="164" t="s">
+      <c r="A37" s="168"/>
+      <c r="H37" s="163"/>
+      <c r="I37" s="163" t="s">
+        <v>158</v>
+      </c>
+      <c r="J37" s="163" t="s">
+        <v>146</v>
+      </c>
+      <c r="K37" s="163" t="s">
+        <v>159</v>
+      </c>
+      <c r="L37" s="163" t="s">
+        <v>160</v>
+      </c>
+      <c r="M37" s="163" t="s">
+        <v>161</v>
+      </c>
+      <c r="N37" s="163" t="s">
+        <v>162</v>
+      </c>
+      <c r="O37" s="163" t="s">
         <v>163</v>
       </c>
-      <c r="J37" s="164" t="s">
-        <v>151</v>
-      </c>
-      <c r="K37" s="164" t="s">
+      <c r="P37" s="163" t="s">
         <v>164</v>
       </c>
-      <c r="L37" s="164" t="s">
-        <v>165</v>
-      </c>
-      <c r="M37" s="164" t="s">
-        <v>166</v>
-      </c>
-      <c r="N37" s="164" t="s">
-        <v>167</v>
-      </c>
-      <c r="O37" s="164" t="s">
-        <v>168</v>
-      </c>
-      <c r="P37" s="164" t="s">
-        <v>169</v>
-      </c>
     </row>
     <row r="38" spans="1:16" ht="16" thickBot="1">
-      <c r="A38" s="168"/>
+      <c r="A38" s="167"/>
       <c r="H38" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="I38">
         <v>903.25547445255484</v>
@@ -15770,7 +15693,7 @@
     </row>
     <row r="39" spans="1:16">
       <c r="H39" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="I39">
         <v>69.769343065693434</v>
@@ -15798,42 +15721,42 @@
       </c>
     </row>
     <row r="40" spans="1:16" ht="15" thickBot="1">
-      <c r="H40" s="163" t="s">
-        <v>171</v>
-      </c>
-      <c r="I40" s="163">
+      <c r="H40" s="162" t="s">
+        <v>166</v>
+      </c>
+      <c r="I40" s="162">
         <v>309.1897810218976</v>
       </c>
-      <c r="J40" s="163">
+      <c r="J40" s="162">
         <v>333.72162042817166</v>
       </c>
-      <c r="K40" s="163">
+      <c r="K40" s="162">
         <v>0.92649011060536257</v>
       </c>
-      <c r="L40" s="163">
+      <c r="L40" s="162">
         <v>0.37245001484419493</v>
       </c>
-      <c r="M40" s="163">
+      <c r="M40" s="162">
         <v>-417.9271671043399</v>
       </c>
-      <c r="N40" s="163">
+      <c r="N40" s="162">
         <v>1036.3067291481352</v>
       </c>
-      <c r="O40" s="163">
+      <c r="O40" s="162">
         <v>-417.9271671043399</v>
       </c>
-      <c r="P40" s="163">
+      <c r="P40" s="162">
         <v>1036.3067291481352</v>
       </c>
     </row>
     <row r="43" spans="1:16">
       <c r="I43" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="44" spans="1:16">
       <c r="I44" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -15853,12 +15776,12 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="26" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="52" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="15" thickBot="1">

</xml_diff>